<commit_message>
Update Liangguang viceroy site with user-verified coordinates and source
</commit_message>
<xml_diff>
--- a/003_Geocoding_and_Validation/geocoding_review.xlsx
+++ b/003_Geocoding_and_Validation/geocoding_review.xlsx
@@ -1740,7 +1740,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>两广总督衙门</t>
+          <t>两广总督衙门旧址（今广东省民政厅）</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1763,28 +1763,40 @@
           <t>site</t>
         </is>
       </c>
-      <c r="H15" s="3" t="n"/>
-      <c r="I15" s="3" t="n"/>
+      <c r="H15" s="3" t="n">
+        <v>23.13196</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>113.26091</v>
+      </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>approximate</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>历史衙门旧址未能可靠确定</t>
-        </is>
-      </c>
-      <c r="L15" s="3" t="n"/>
-      <c r="M15" s="3" t="n"/>
+          <t>广州市越华路118号现今旧址（广东省民政厅）近似点</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yuexiu.gov.cn/data/cms/category/xzzfsj/kejj1548668945490809.pdf</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yuexiu.gov.cn/data/cms/category/xzzfsj/kejj1548668945490809.pdf</t>
+        </is>
+      </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>现今旧址由用户核实；历史建筑边界／到访日期仍需核验</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
-          <t>对“两广总督署／两广总督衙门”的OSM检索均未返回匹配；未取得可核查、可地理配准的旧址史料或历史地图。不能把机构条目、城市中心或其他时期衙门替作1880年代到访建筑，故坐标保持null。</t>
+          <t>按用户提供的已核实资料，对应广州市越华路118号，今广东省民政厅；采用用户提供的23.13196、113.26091作为现今旧址的近似定位，来源为越秀区政府PDF。不是历史衙门建筑轮廓的精确坐标，也不据此补写到访日期或确认旅行连线。</t>
         </is>
       </c>
       <c r="P15" s="3" t="inlineStr">
@@ -1797,7 +1809,11 @@
           <t>仅保留原笔记分组日期，缺日期则不补。不得以sequence或坐标存在推定已确认到访顺序。</t>
         </is>
       </c>
-      <c r="R15" s="3" t="n"/>
+      <c r="R15" s="3" t="inlineStr">
+        <is>
+          <t>沿用数据集WGS84约定；坐标系未独立核验</t>
+        </is>
+      </c>
       <c r="S15" s="3" t="inlineStr">
         <is>
           <t>2026-10-12</t>
@@ -1843,7 +1859,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>001_最新版Excel替换_重新编号_坐标核验/places_authoritative.xlsx；SHA256=f8dcb5f710664716dfa4c5c67828178af47fced517abfeb60d807ca245191197</t>
+          <t>001_最新版Excel替换_重新编号_坐标核验/places_authoritative.xlsx；SHA256=f8dcb5f710664716dfa4c5c67828178af47fced517abfeb60d807ca245191197；P031另按用户本次提供的已核实名称、现今旧址坐标及来源更新。</t>
         </is>
       </c>
     </row>
@@ -1867,7 +1883,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>5条city-level，6条approximate，2条exact，1条unknown。</t>
+          <t>5条city-level，7条approximate，2条exact；14条均有坐标和来源。</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1931,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>本轮不确认任何相邻点旅行连线；尤其节庆对应、城市概览、区域范围、日期缺失及衙门未识别不能直接连成亲历路线。</t>
+          <t>不确认任何相邻点旅行连线；城市概览、历史区域范围及缺日期记录不能直接连成亲历路线。P031现今旧址已由用户核实，但日期与历史建筑边界未补写。</t>
         </is>
       </c>
     </row>

</xml_diff>